<commit_message>
Import event reminder feature from MiniCRM
</commit_message>
<xml_diff>
--- a/assets/templates/lead_upload_template.xlsx
+++ b/assets/templates/lead_upload_template.xlsx
@@ -1,105 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dfcc2c3ff10d4ab1/Documents/lead_capture_crm/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{002A7AA4-2BF2-467F-A14C-9D0413926F77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8EBB88D-B47D-4673-BFA5-03E3F1E663B1}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lead Upload" sheetId="1" r:id="rId1"/>
+    <sheet name="Lead Upload" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>Lead Name</t>
-  </si>
-  <si>
-    <t>Lead Email</t>
-  </si>
-  <si>
-    <t>Lead Source</t>
-  </si>
-  <si>
-    <t>Lead Category</t>
-  </si>
-  <si>
-    <t>Lead Priority</t>
-  </si>
-  <si>
-    <t>Lead Value</t>
-  </si>
-  <si>
-    <t>Lead Status</t>
-  </si>
-  <si>
-    <t>Company Name</t>
-  </si>
-  <si>
-    <t>Company Mobile</t>
-  </si>
-  <si>
-    <t>Country</t>
-  </si>
-  <si>
-    <t>State</t>
-  </si>
-  <si>
-    <t>City</t>
-  </si>
-  <si>
-    <t>Address</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1A56DB"/>
-        <bgColor rgb="FF1A56DB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor rgb="FF1A56DB"/>
+        <fgColor rgb="001A56DB"/>
+        <bgColor rgb="001A56DB"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,45 +55,100 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="00D1D5DB"/>
       </left>
       <right style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="00D1D5DB"/>
       </right>
       <top style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="00D1D5DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="00D1D5DB"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -439,68 +436,107 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="4" width="15" customWidth="1"/>
-    <col min="5" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="22" customWidth="1"/>
-    <col min="14" max="14" width="25" customWidth="1"/>
-    <col min="15" max="15" width="22" customWidth="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="2"/>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Lead Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Lead Email</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Lead Source</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Lead Category</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Lead Priority</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Lead Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Lead Status</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Company Name</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Company Mobile</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Created At (dd-MM-yyyy)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>